<commit_message>
Add Quickbooks sync, Vendor View of the Dashboard
</commit_message>
<xml_diff>
--- a/Vendor Database_Payments & Tracking/Sample Platform Reports by Platform/US Arcades_ViewTime Royalty Statement_July 2025_8-6-25.xlsx
+++ b/Vendor Database_Payments & Tracking/Sample Platform Reports by Platform/US Arcades_ViewTime Royalty Statement_July 2025_8-6-25.xlsx
@@ -1,25 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment authorId="0" ref="G13">
+    <comment ref="G13" authorId="0">
       <text>
-        <t xml:space="preserve">Can add these in manually each month before uploading
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="SimSun"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">Can add these in manually each month before uploading
 </t>
+        </r>
       </text>
     </comment>
   </commentList>
@@ -34,28 +57,31 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="13"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Helvetica Neue"/>
-        <b/>
-        <color rgb="FF1F1F1F"/>
-        <sz val="13.0"/>
+        <charset val="134"/>
       </rPr>
       <t>"US Arcades - DO NOT REPLY"</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="13"/>
+        <color rgb="FF5F6368"/>
         <rFont val="Helvetica"/>
-        <b/>
-        <color rgb="FF5F6368"/>
-        <sz val="13.0"/>
+        <charset val="134"/>
       </rPr>
       <t> </t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="13"/>
+        <color rgb="FF5E5E5E"/>
         <rFont val="Helvetica"/>
-        <b/>
-        <color rgb="FF5E5E5E"/>
-        <sz val="13.0"/>
+        <charset val="134"/>
       </rPr>
       <t>&lt;alerter@usarcades.com&gt;</t>
     </r>
@@ -190,84 +216,269 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="13">
-    <font>
-      <sz val="12.0"/>
+  <fonts count="35">
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="18.0"/>
+      <sz val="18"/>
       <color rgb="FF1F1F1F"/>
       <name val="Helvetica Neue"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="13.0"/>
+      <sz val="13"/>
       <color rgb="FF1F1F1F"/>
       <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF5E5E5E"/>
       <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF222222"/>
       <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF444444"/>
       <name val="Helvetica Neue"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Verdana"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Verdana"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Verdana"/>
-    </font>
-    <font>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF5F6368"/>
+      <name val="Helvetica"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF5E5E5E"/>
+      <name val="Helvetica"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="SimSun"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -275,67 +486,771 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
-    <border/>
+  <borders count="11">
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="26">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="0" fontId="11" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="7" numFmtId="3" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="2" fillId="0" fontId="7" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="2" fillId="0" fontId="11" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="3" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color theme="4"/>
+        </left>
+        <right style="thin">
+          <color theme="4"/>
+        </right>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <horizontal style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    </tableStyle>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
@@ -346,16 +1261,20 @@
     <xdr:ext cx="9525" cy="9525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.gif"/>
+        <xdr:cNvPr id="2" name="image1.gif"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
+        <a:blip r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5182235" y="200025"/>
+          <a:ext cx="9525" cy="9525"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -368,7 +1287,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -558,29 +1477,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G1000"/>
+  <sheetFormatPr defaultColWidth="11.2166666666667" defaultRowHeight="15" customHeight="1" outlineLevelCol="6"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="41.78"/>
-    <col customWidth="1" min="2" max="2" width="10.56"/>
-    <col customWidth="1" min="3" max="3" width="15.67"/>
-    <col customWidth="1" min="4" max="4" width="12.11"/>
-    <col customWidth="1" min="5" max="26" width="10.56"/>
+    <col min="1" max="1" width="41.7833333333333" customWidth="1"/>
+    <col min="2" max="2" width="10.5583333333333" customWidth="1"/>
+    <col min="3" max="3" width="15.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="12.1083333333333" customWidth="1"/>
+    <col min="5" max="26" width="10.5583333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
+    <row r="2" ht="15.75" customHeight="1" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -593,13 +1512,13 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1"/>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" ht="15.75" customHeight="1" spans="1:1">
       <c r="A4" s="3" t="e">
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1"/>
-    <row r="6" ht="15.75" customHeight="1">
+    <row r="6" ht="15.75" customHeight="1" spans="1:2">
       <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
@@ -607,23 +1526,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
+    <row r="7" ht="15.75" customHeight="1" spans="1:1">
       <c r="A7" s="7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" ht="15.75" customHeight="1" spans="1:1">
       <c r="A8" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" ht="15.75" customHeight="1" spans="1:1">
       <c r="A9" s="7"/>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" ht="15.75" customHeight="1" spans="1:1">
       <c r="A10" s="7"/>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" ht="15.75" customHeight="1" spans="1:2">
       <c r="A11" s="7" t="s">
         <v>6</v>
       </c>
@@ -631,10 +1550,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" ht="15.75" customHeight="1" spans="1:1">
       <c r="A12" s="7"/>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" ht="15.75" customHeight="1" spans="1:7">
       <c r="A13" s="9" t="s">
         <v>8</v>
       </c>
@@ -651,63 +1570,63 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" ht="15.75" customHeight="1" spans="1:1">
       <c r="A14" s="11"/>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" ht="15.75" customHeight="1" spans="1:1">
       <c r="A15" s="12"/>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
+    <row r="16" ht="15.75" customHeight="1" spans="1:4">
       <c r="A16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="7">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="C16" s="13">
-        <v>612775.0</v>
+        <v>612775</v>
       </c>
       <c r="D16" s="14">
         <v>57.56</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" ht="15.75" customHeight="1" spans="1:4">
       <c r="A17" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B17" s="7">
-        <v>54.0</v>
+        <v>54</v>
       </c>
       <c r="C17" s="13">
-        <v>1303091.0</v>
+        <v>1303091</v>
       </c>
       <c r="D17" s="14">
         <v>122.15</v>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
+    <row r="18" ht="15.75" customHeight="1" spans="1:4">
       <c r="A18" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="7">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C18" s="13">
-        <v>91538.0</v>
+        <v>91538</v>
       </c>
       <c r="D18" s="14">
         <v>9.21</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="15.75" customHeight="1" spans="1:6">
       <c r="A19" s="15" t="s">
         <v>16</v>
       </c>
       <c r="B19" s="15">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="C19" s="16">
-        <v>332846.0</v>
+        <v>332846</v>
       </c>
       <c r="D19" s="17">
         <v>31.33</v>
@@ -719,127 +1638,127 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1" spans="1:4">
       <c r="A20" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="7">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="C20" s="13">
-        <v>519153.0</v>
+        <v>519153</v>
       </c>
       <c r="D20" s="14">
         <v>48.37</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1" spans="1:4">
       <c r="A21" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="7">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C21" s="13">
-        <v>219630.0</v>
+        <v>219630</v>
       </c>
       <c r="D21" s="14">
         <v>20.29</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1" spans="1:4">
       <c r="A22" s="7" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C22" s="13">
-        <v>222094.0</v>
+        <v>222094</v>
       </c>
       <c r="D22" s="14">
         <v>21.51</v>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1" spans="1:4">
       <c r="A23" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C23" s="13">
-        <v>33883.0</v>
+        <v>33883</v>
       </c>
       <c r="D23" s="14">
         <v>3.02</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1" spans="1:4">
       <c r="A24" s="7" t="s">
         <v>22</v>
       </c>
       <c r="B24" s="7">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C24" s="13">
-        <v>357026.0</v>
+        <v>357026</v>
       </c>
       <c r="D24" s="14">
         <v>34.24</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" ht="15.75" customHeight="1" spans="1:4">
       <c r="A25" s="7" t="s">
         <v>23</v>
       </c>
       <c r="B25" s="7">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C25" s="13">
-        <v>73491.0</v>
+        <v>73491</v>
       </c>
       <c r="D25" s="14">
         <v>6.57</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" ht="15.75" customHeight="1" spans="1:4">
       <c r="A26" s="7" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="7">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="C26" s="13">
-        <v>684170.0</v>
+        <v>684170</v>
       </c>
       <c r="D26" s="14">
         <v>63.42</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" ht="15.75" customHeight="1" spans="1:4">
       <c r="A27" s="7" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="7">
-        <v>39.0</v>
+        <v>39</v>
       </c>
       <c r="C27" s="13">
-        <v>715476.0</v>
+        <v>715476</v>
       </c>
       <c r="D27" s="14">
         <v>66.54</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="15.75" customHeight="1" spans="1:6">
       <c r="A28" s="15" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="15">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C28" s="16">
-        <v>141548.0</v>
+        <v>141548</v>
       </c>
       <c r="D28" s="17">
         <v>13.96</v>
@@ -851,43 +1770,43 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1" spans="1:4">
       <c r="A29" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="7">
-        <v>33.0</v>
+        <v>33</v>
       </c>
       <c r="C29" s="13">
-        <v>1178734.0</v>
+        <v>1178734</v>
       </c>
       <c r="D29" s="14">
         <v>113.14</v>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" ht="15.75" customHeight="1" spans="1:4">
       <c r="A30" s="7" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="7">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="13">
-        <v>7061.0</v>
+        <v>7061</v>
       </c>
       <c r="D30" s="14">
         <v>0.65</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1" spans="1:6">
       <c r="A31" s="15" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="15">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C31" s="16">
-        <v>6360.0</v>
+        <v>6360</v>
       </c>
       <c r="D31" s="17">
         <v>0.54</v>
@@ -899,15 +1818,15 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="15.75" customHeight="1" spans="1:6">
       <c r="A32" s="20" t="s">
         <v>32</v>
       </c>
       <c r="B32" s="20">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="C32" s="21">
-        <v>369497.0</v>
+        <v>369497</v>
       </c>
       <c r="D32" s="22">
         <v>34.1</v>
@@ -919,29 +1838,29 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="15.75" customHeight="1" spans="1:4">
       <c r="A33" s="7" t="s">
         <v>33</v>
       </c>
       <c r="B33" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="C33" s="13">
-        <v>175034.0</v>
+        <v>175034</v>
       </c>
       <c r="D33" s="14">
         <v>17.45</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" ht="15.75" customHeight="1" spans="1:6">
       <c r="A34" s="15" t="s">
         <v>34</v>
       </c>
       <c r="B34" s="15">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C34" s="16">
-        <v>41071.0</v>
+        <v>41071</v>
       </c>
       <c r="D34" s="17">
         <v>3.95</v>
@@ -953,43 +1872,43 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" ht="15.75" customHeight="1" spans="1:4">
       <c r="A35" s="7" t="s">
         <v>36</v>
       </c>
       <c r="B35" s="7">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="C35" s="13">
-        <v>824075.0</v>
+        <v>824075</v>
       </c>
       <c r="D35" s="14">
         <v>78.13</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" ht="15.75" customHeight="1" spans="1:4">
       <c r="A36" s="7" t="s">
         <v>37</v>
       </c>
       <c r="B36" s="7">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="C36" s="13">
-        <v>291622.0</v>
+        <v>291622</v>
       </c>
       <c r="D36" s="14">
         <v>27.47</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="15.75" customHeight="1" spans="1:6">
       <c r="A37" s="15" t="s">
         <v>38</v>
       </c>
       <c r="B37" s="15">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C37" s="16">
-        <v>4338.0</v>
+        <v>4338</v>
       </c>
       <c r="D37" s="17">
         <v>0.41</v>
@@ -1001,15 +1920,15 @@
         <v>39</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="15.75" customHeight="1" spans="1:6">
       <c r="A38" s="20" t="s">
         <v>40</v>
       </c>
       <c r="B38" s="20">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="C38" s="21">
-        <v>7625.0</v>
+        <v>7625</v>
       </c>
       <c r="D38" s="22">
         <v>0.7</v>
@@ -1021,15 +1940,15 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="15.75" customHeight="1" spans="1:6">
       <c r="A39" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B39" s="7">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C39" s="13">
-        <v>232314.0</v>
+        <v>232314</v>
       </c>
       <c r="D39" s="14">
         <v>21.96</v>
@@ -1041,29 +1960,29 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" ht="15.75" customHeight="1" spans="1:4">
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="13"/>
       <c r="D40" s="14"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="15.75" customHeight="1" spans="1:1">
       <c r="A41" s="11"/>
     </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="15.75" customHeight="1" spans="1:1">
       <c r="A44" s="12"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="15.75" customHeight="1" spans="1:4">
       <c r="A45" s="9" t="s">
         <v>43</v>
       </c>
       <c r="B45" s="9">
-        <v>290.0</v>
+        <v>290</v>
       </c>
       <c r="C45" s="24">
-        <v>8444452.0</v>
+        <v>8444452</v>
       </c>
       <c r="D45" s="25">
         <v>796.65</v>
@@ -2027,20 +2946,20 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A41:A44"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A41:A44"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId2" ref="A8"/>
+    <hyperlink ref="A8" r:id="rId4" display="stacey@rldd.com"/>
   </hyperlinks>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="1" orientation="landscape"/>
+  <headerFooter/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>